<commit_message>
GBDS JUNE & JULY 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JULY FILES 2026/BAL 2 ENC CAL JUNE-JULY.xlsx
+++ b/GBDS JULY FILES 2026/BAL 2 ENC CAL JUNE-JULY.xlsx
@@ -5,20 +5,20 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JUNE FILES 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JULY FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60AF82A1-309E-416A-9B6B-A9FB1699CD50}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E03EC2E-EEA6-48E0-98F4-7690CA817C11}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BAL 2 ENC CAL" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="BAL 2 ENC CAL BERLYN" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'BAL 2 ENC CAL'!$N$1:$X$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'BAL 2 ENC CAL'!$A$1:$N$48</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'BAL 2 ENC CAL BERLYN'!$A$1:$N$48</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="63">
   <si>
     <t>SKU</t>
   </si>
@@ -218,14 +218,17 @@
     <t>HTA</t>
   </si>
   <si>
-    <t>KIRIN CAN</t>
+    <t>BALANCE TO ENCODE</t>
+  </si>
+  <si>
+    <t>ENDING ENVENTORY</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -264,8 +267,30 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="28"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -328,8 +353,36 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
@@ -342,10 +395,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
@@ -384,35 +443,44 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="5"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="4" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="3" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="0" xfId="5" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="5" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="6" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -420,15 +488,53 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="5" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" xfId="5" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="7">
+    <cellStyle name="20% - Accent4" xfId="5" builtinId="42"/>
+    <cellStyle name="40% - Accent1" xfId="1" builtinId="31"/>
+    <cellStyle name="40% - Accent3" xfId="3" builtinId="39"/>
+    <cellStyle name="40% - Accent4" xfId="6" builtinId="43"/>
+    <cellStyle name="Accent2" xfId="2" builtinId="33"/>
+    <cellStyle name="Accent4" xfId="4" builtinId="41"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFCC99FF"/>
+      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3E0E37"/>
+      <color rgb="FF5F035B"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -802,19 +908,19 @@
       </c>
       <c r="M1" s="2"/>
       <c r="N1" s="12"/>
-      <c r="O1" s="24" t="s">
+      <c r="O1" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
+      <c r="P1" s="34"/>
+      <c r="Q1" s="34"/>
+      <c r="R1" s="34"/>
       <c r="S1" s="12"/>
-      <c r="T1" s="24" t="s">
+      <c r="T1" s="34" t="s">
         <v>42</v>
       </c>
-      <c r="U1" s="24"/>
-      <c r="V1" s="24"/>
-      <c r="W1" s="24"/>
+      <c r="U1" s="34"/>
+      <c r="V1" s="34"/>
+      <c r="W1" s="34"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
@@ -842,10 +948,10 @@
         <v>1</v>
       </c>
       <c r="N2" s="12"/>
-      <c r="O2" s="26" t="s">
+      <c r="O2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="P2" s="27"/>
+      <c r="P2" s="36"/>
       <c r="Q2" s="4" t="s">
         <v>1</v>
       </c>
@@ -853,10 +959,10 @@
         <v>26</v>
       </c>
       <c r="S2" s="12"/>
-      <c r="T2" s="26" t="s">
+      <c r="T2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="U2" s="27"/>
+      <c r="U2" s="36"/>
       <c r="V2" s="4" t="s">
         <v>1</v>
       </c>
@@ -884,35 +990,31 @@
       </c>
       <c r="M3" s="10"/>
       <c r="N3" s="12"/>
-      <c r="O3" s="22" t="s">
+      <c r="O3" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="P3" s="22"/>
-      <c r="Q3" s="10">
-        <v>3</v>
-      </c>
-      <c r="R3" s="25">
+      <c r="P3" s="32"/>
+      <c r="Q3" s="10"/>
+      <c r="R3" s="37">
         <f>SUM(Q3:Q47)</f>
-        <v>49275</v>
+        <v>0</v>
       </c>
       <c r="S3" s="12"/>
-      <c r="T3" s="22" t="s">
+      <c r="T3" s="32" t="s">
         <v>31</v>
       </c>
-      <c r="U3" s="22"/>
+      <c r="U3" s="32"/>
       <c r="V3" s="10"/>
-      <c r="W3" s="25">
+      <c r="W3" s="37">
         <f>SUM(V3:V47)</f>
-        <v>2143</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="18">
-        <v>1</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="B4" s="10"/>
       <c r="F4" s="5" t="s">
         <v>2</v>
       </c>
@@ -928,21 +1030,19 @@
       </c>
       <c r="M4" s="10"/>
       <c r="N4" s="12"/>
-      <c r="O4" s="22" t="s">
+      <c r="O4" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="10">
-        <v>4</v>
-      </c>
-      <c r="R4" s="25"/>
+      <c r="P4" s="32"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="37"/>
       <c r="S4" s="12"/>
-      <c r="T4" s="22" t="s">
+      <c r="T4" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="U4" s="22"/>
+      <c r="U4" s="32"/>
       <c r="V4" s="10"/>
-      <c r="W4" s="25"/>
+      <c r="W4" s="37"/>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -950,11 +1050,9 @@
       </c>
       <c r="B5" s="10"/>
       <c r="F5" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="G5" s="10">
-        <v>1</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="G5" s="10"/>
       <c r="H5" s="12"/>
       <c r="I5" s="5" t="s">
         <v>45</v>
@@ -966,21 +1064,19 @@
       </c>
       <c r="M5" s="10"/>
       <c r="N5" s="12"/>
-      <c r="O5" s="22" t="s">
+      <c r="O5" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="10">
-        <v>1</v>
-      </c>
-      <c r="R5" s="25"/>
+      <c r="P5" s="32"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="37"/>
       <c r="S5" s="12"/>
-      <c r="T5" s="22" t="s">
+      <c r="T5" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="U5" s="22"/>
+      <c r="U5" s="32"/>
       <c r="V5" s="10"/>
-      <c r="W5" s="25"/>
+      <c r="W5" s="37"/>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
@@ -1002,21 +1098,19 @@
       </c>
       <c r="M6" s="10"/>
       <c r="N6" s="12"/>
-      <c r="O6" s="22" t="s">
+      <c r="O6" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="P6" s="22"/>
-      <c r="Q6" s="10">
-        <v>1</v>
-      </c>
-      <c r="R6" s="25"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="37"/>
       <c r="S6" s="12"/>
-      <c r="T6" s="22" t="s">
+      <c r="T6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="U6" s="22"/>
+      <c r="U6" s="32"/>
       <c r="V6" s="10"/>
-      <c r="W6" s="25"/>
+      <c r="W6" s="37"/>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
@@ -1038,27 +1132,23 @@
       </c>
       <c r="M7" s="10"/>
       <c r="N7" s="12"/>
-      <c r="O7" s="22" t="s">
+      <c r="O7" s="32" t="s">
         <v>50</v>
       </c>
-      <c r="P7" s="22"/>
-      <c r="Q7" s="10">
-        <v>4</v>
-      </c>
-      <c r="R7" s="25"/>
+      <c r="P7" s="32"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="37"/>
       <c r="S7" s="12"/>
       <c r="T7" s="15"/>
       <c r="U7" s="15"/>
       <c r="V7" s="10"/>
-      <c r="W7" s="25"/>
+      <c r="W7" s="37"/>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="18">
-        <v>1</v>
-      </c>
+      <c r="B8" s="10"/>
       <c r="F8" s="5" t="s">
         <v>33</v>
       </c>
@@ -1074,21 +1164,19 @@
       </c>
       <c r="M8" s="10"/>
       <c r="N8" s="12"/>
-      <c r="O8" s="22" t="s">
+      <c r="O8" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="10">
-        <v>3</v>
-      </c>
-      <c r="R8" s="25"/>
+      <c r="P8" s="32"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="37"/>
       <c r="S8" s="12"/>
-      <c r="T8" s="22" t="s">
+      <c r="T8" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="U8" s="22"/>
+      <c r="U8" s="32"/>
       <c r="V8" s="10"/>
-      <c r="W8" s="25"/>
+      <c r="W8" s="37"/>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
@@ -1098,9 +1186,7 @@
       <c r="F9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="G9" s="10">
-        <v>1</v>
-      </c>
+      <c r="G9" s="10"/>
       <c r="H9" s="12"/>
       <c r="I9" s="5" t="s">
         <v>51</v>
@@ -1112,21 +1198,19 @@
       </c>
       <c r="M9" s="10"/>
       <c r="N9" s="12"/>
-      <c r="O9" s="22" t="s">
+      <c r="O9" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="P9" s="22"/>
-      <c r="Q9" s="10">
-        <v>6</v>
-      </c>
-      <c r="R9" s="25"/>
+      <c r="P9" s="32"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="37"/>
       <c r="S9" s="12"/>
-      <c r="T9" s="22" t="s">
+      <c r="T9" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="U9" s="22"/>
+      <c r="U9" s="32"/>
       <c r="V9" s="10"/>
-      <c r="W9" s="25"/>
+      <c r="W9" s="37"/>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
@@ -1148,27 +1232,23 @@
       </c>
       <c r="M10" s="10"/>
       <c r="N10" s="12"/>
-      <c r="O10" s="22" t="s">
+      <c r="O10" s="32" t="s">
         <v>51</v>
       </c>
-      <c r="P10" s="22"/>
-      <c r="Q10" s="10">
-        <v>3</v>
-      </c>
-      <c r="R10" s="25"/>
+      <c r="P10" s="32"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="37"/>
       <c r="S10" s="12"/>
       <c r="T10" s="13"/>
       <c r="U10" s="13"/>
       <c r="V10" s="10"/>
-      <c r="W10" s="25"/>
+      <c r="W10" s="37"/>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B11" s="18">
-        <v>1</v>
-      </c>
+      <c r="B11" s="10"/>
       <c r="F11" s="5" t="s">
         <v>4</v>
       </c>
@@ -1184,35 +1264,29 @@
       </c>
       <c r="M11" s="10"/>
       <c r="N11" s="12"/>
-      <c r="O11" s="22" t="s">
+      <c r="O11" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="P11" s="22"/>
-      <c r="Q11" s="10">
-        <v>1</v>
-      </c>
-      <c r="R11" s="25"/>
+      <c r="P11" s="32"/>
+      <c r="Q11" s="10"/>
+      <c r="R11" s="37"/>
       <c r="S11" s="12"/>
-      <c r="T11" s="22" t="s">
+      <c r="T11" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="U11" s="22"/>
+      <c r="U11" s="32"/>
       <c r="V11" s="10"/>
-      <c r="W11" s="25"/>
+      <c r="W11" s="37"/>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="18">
-        <v>30</v>
-      </c>
+      <c r="B12" s="10"/>
       <c r="F12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="G12" s="10">
-        <v>1</v>
-      </c>
+      <c r="G12" s="10"/>
       <c r="H12" s="12"/>
       <c r="I12" s="5" t="s">
         <v>43</v>
@@ -1224,19 +1298,17 @@
       </c>
       <c r="M12" s="10"/>
       <c r="N12" s="12"/>
-      <c r="O12" s="22" t="s">
+      <c r="O12" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="P12" s="22"/>
-      <c r="Q12" s="10">
-        <v>9</v>
-      </c>
-      <c r="R12" s="25"/>
+      <c r="P12" s="32"/>
+      <c r="Q12" s="10"/>
+      <c r="R12" s="37"/>
       <c r="S12" s="12"/>
       <c r="T12" s="13"/>
       <c r="U12" s="13"/>
       <c r="V12" s="10"/>
-      <c r="W12" s="25"/>
+      <c r="W12" s="37"/>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
@@ -1246,49 +1318,37 @@
       <c r="F13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="10">
-        <v>10</v>
-      </c>
+      <c r="G13" s="10"/>
       <c r="H13" s="12"/>
       <c r="I13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="J13" s="10">
-        <v>10</v>
-      </c>
+      <c r="J13" s="10"/>
       <c r="K13" s="12"/>
       <c r="L13" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M13" s="10">
-        <v>10</v>
-      </c>
+      <c r="M13" s="10"/>
       <c r="N13" s="12"/>
-      <c r="O13" s="22" t="s">
+      <c r="O13" s="32" t="s">
         <v>5</v>
       </c>
-      <c r="P13" s="22"/>
-      <c r="Q13" s="10">
-        <v>124</v>
-      </c>
-      <c r="R13" s="25"/>
+      <c r="P13" s="32"/>
+      <c r="Q13" s="10"/>
+      <c r="R13" s="37"/>
       <c r="S13" s="12"/>
-      <c r="T13" s="22" t="s">
+      <c r="T13" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="U13" s="22"/>
-      <c r="V13" s="10">
-        <v>63</v>
-      </c>
-      <c r="W13" s="25"/>
+      <c r="U13" s="32"/>
+      <c r="V13" s="10"/>
+      <c r="W13" s="37"/>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B14" s="18">
-        <v>70</v>
-      </c>
+      <c r="B14" s="10"/>
       <c r="F14" s="5" t="s">
         <v>6</v>
       </c>
@@ -1304,21 +1364,19 @@
       </c>
       <c r="M14" s="10"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="22" t="s">
+      <c r="O14" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="P14" s="22"/>
-      <c r="Q14" s="10">
-        <v>0</v>
-      </c>
-      <c r="R14" s="25"/>
+      <c r="P14" s="32"/>
+      <c r="Q14" s="10"/>
+      <c r="R14" s="37"/>
       <c r="S14" s="12"/>
-      <c r="T14" s="22" t="s">
+      <c r="T14" s="32" t="s">
         <v>6</v>
       </c>
-      <c r="U14" s="22"/>
+      <c r="U14" s="32"/>
       <c r="V14" s="10"/>
-      <c r="W14" s="25"/>
+      <c r="W14" s="37"/>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
@@ -1328,41 +1386,31 @@
       <c r="F15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G15" s="10">
-        <v>24</v>
-      </c>
+      <c r="G15" s="10"/>
       <c r="H15" s="12"/>
       <c r="I15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="J15" s="10">
-        <v>23</v>
-      </c>
+      <c r="J15" s="10"/>
       <c r="K15" s="12"/>
       <c r="L15" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="M15" s="10">
-        <v>23</v>
-      </c>
+      <c r="M15" s="10"/>
       <c r="N15" s="12"/>
-      <c r="O15" s="22" t="s">
+      <c r="O15" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="10">
-        <v>2</v>
-      </c>
-      <c r="R15" s="25"/>
+      <c r="P15" s="32"/>
+      <c r="Q15" s="10"/>
+      <c r="R15" s="37"/>
       <c r="S15" s="12"/>
-      <c r="T15" s="22" t="s">
+      <c r="T15" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="U15" s="22"/>
-      <c r="V15" s="10">
-        <v>28</v>
-      </c>
-      <c r="W15" s="25"/>
+      <c r="U15" s="32"/>
+      <c r="V15" s="10"/>
+      <c r="W15" s="37"/>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
@@ -1384,21 +1432,19 @@
       </c>
       <c r="M16" s="10"/>
       <c r="N16" s="12"/>
-      <c r="O16" s="22" t="s">
+      <c r="O16" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="P16" s="22"/>
-      <c r="Q16" s="10">
-        <v>60</v>
-      </c>
-      <c r="R16" s="25"/>
+      <c r="P16" s="32"/>
+      <c r="Q16" s="10"/>
+      <c r="R16" s="37"/>
       <c r="S16" s="12"/>
-      <c r="T16" s="22" t="s">
+      <c r="T16" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="U16" s="22"/>
+      <c r="U16" s="32"/>
       <c r="V16" s="10"/>
-      <c r="W16" s="25"/>
+      <c r="W16" s="37"/>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
@@ -1420,29 +1466,25 @@
       </c>
       <c r="M17" s="10"/>
       <c r="N17" s="12"/>
-      <c r="O17" s="22" t="s">
+      <c r="O17" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="10">
-        <v>0</v>
-      </c>
-      <c r="R17" s="25"/>
+      <c r="P17" s="32"/>
+      <c r="Q17" s="10"/>
+      <c r="R17" s="37"/>
       <c r="S17" s="12"/>
-      <c r="T17" s="22" t="s">
+      <c r="T17" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="U17" s="22"/>
+      <c r="U17" s="32"/>
       <c r="V17" s="10"/>
-      <c r="W17" s="25"/>
+      <c r="W17" s="37"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="18">
-        <v>2</v>
-      </c>
+      <c r="B18" s="10"/>
       <c r="F18" s="5" t="s">
         <v>36</v>
       </c>
@@ -1458,29 +1500,25 @@
       </c>
       <c r="M18" s="10"/>
       <c r="N18" s="12"/>
-      <c r="O18" s="22" t="s">
+      <c r="O18" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="P18" s="22"/>
-      <c r="Q18" s="10">
-        <v>63</v>
-      </c>
-      <c r="R18" s="25"/>
+      <c r="P18" s="32"/>
+      <c r="Q18" s="10"/>
+      <c r="R18" s="37"/>
       <c r="S18" s="12"/>
-      <c r="T18" s="22" t="s">
+      <c r="T18" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="U18" s="22"/>
+      <c r="U18" s="32"/>
       <c r="V18" s="10"/>
-      <c r="W18" s="25"/>
+      <c r="W18" s="37"/>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="18">
-        <v>1</v>
-      </c>
+      <c r="B19" s="10"/>
       <c r="F19" s="5" t="s">
         <v>10</v>
       </c>
@@ -1489,46 +1527,36 @@
       <c r="I19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="J19" s="10">
-        <v>1</v>
-      </c>
+      <c r="J19" s="10"/>
       <c r="K19" s="12"/>
       <c r="L19" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M19" s="10">
-        <v>1</v>
-      </c>
+      <c r="M19" s="10"/>
       <c r="N19" s="12"/>
-      <c r="O19" s="22" t="s">
+      <c r="O19" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="P19" s="22"/>
-      <c r="Q19" s="10">
-        <v>6</v>
-      </c>
-      <c r="R19" s="25"/>
+      <c r="P19" s="32"/>
+      <c r="Q19" s="10"/>
+      <c r="R19" s="37"/>
       <c r="S19" s="12"/>
-      <c r="T19" s="22" t="s">
+      <c r="T19" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="U19" s="22"/>
+      <c r="U19" s="32"/>
       <c r="V19" s="10"/>
-      <c r="W19" s="25"/>
+      <c r="W19" s="37"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="18">
-        <v>16</v>
-      </c>
+      <c r="B20" s="10"/>
       <c r="F20" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="G20" s="10">
-        <v>1</v>
-      </c>
+      <c r="G20" s="10"/>
       <c r="H20" s="12"/>
       <c r="I20" s="5" t="s">
         <v>37</v>
@@ -1540,35 +1568,29 @@
       </c>
       <c r="M20" s="10"/>
       <c r="N20" s="12"/>
-      <c r="O20" s="22" t="s">
+      <c r="O20" s="32" t="s">
         <v>10</v>
       </c>
-      <c r="P20" s="22"/>
-      <c r="Q20" s="10">
-        <v>15</v>
-      </c>
-      <c r="R20" s="25"/>
+      <c r="P20" s="32"/>
+      <c r="Q20" s="10"/>
+      <c r="R20" s="37"/>
       <c r="S20" s="12"/>
-      <c r="T20" s="22" t="s">
+      <c r="T20" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="U20" s="22"/>
+      <c r="U20" s="32"/>
       <c r="V20" s="10"/>
-      <c r="W20" s="25"/>
+      <c r="W20" s="37"/>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B21" s="18">
-        <v>209</v>
-      </c>
+      <c r="B21" s="10"/>
       <c r="F21" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="10">
-        <v>16</v>
-      </c>
+      <c r="G21" s="10"/>
       <c r="H21" s="12"/>
       <c r="I21" s="5" t="s">
         <v>11</v>
@@ -1580,65 +1602,53 @@
       </c>
       <c r="M21" s="10"/>
       <c r="N21" s="12"/>
-      <c r="O21" s="22" t="s">
+      <c r="O21" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="P21" s="22"/>
-      <c r="Q21" s="10">
-        <v>2</v>
-      </c>
-      <c r="R21" s="25"/>
+      <c r="P21" s="32"/>
+      <c r="Q21" s="10"/>
+      <c r="R21" s="37"/>
       <c r="S21" s="12"/>
-      <c r="T21" s="22" t="s">
+      <c r="T21" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="U21" s="22"/>
+      <c r="U21" s="32"/>
       <c r="V21" s="10"/>
-      <c r="W21" s="25"/>
+      <c r="W21" s="37"/>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="18">
-        <v>1</v>
-      </c>
+      <c r="B22" s="10"/>
       <c r="F22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="G22" s="10">
-        <v>70</v>
-      </c>
+      <c r="G22" s="10"/>
       <c r="H22" s="12"/>
       <c r="I22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="J22" s="10">
-        <v>70</v>
-      </c>
+      <c r="J22" s="10"/>
       <c r="K22" s="12"/>
       <c r="L22" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="M22" s="10">
-        <v>69</v>
-      </c>
+      <c r="M22" s="10"/>
       <c r="N22" s="12"/>
-      <c r="O22" s="22" t="s">
+      <c r="O22" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="P22" s="22"/>
-      <c r="Q22" s="10">
-        <v>90</v>
-      </c>
-      <c r="R22" s="25"/>
+      <c r="P22" s="32"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="37"/>
       <c r="S22" s="12"/>
-      <c r="T22" s="22" t="s">
+      <c r="T22" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="U22" s="22"/>
+      <c r="U22" s="32"/>
       <c r="V22" s="10"/>
-      <c r="W22" s="25"/>
+      <c r="W22" s="37"/>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
@@ -1648,9 +1658,7 @@
       <c r="F23" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="10">
-        <v>1</v>
-      </c>
+      <c r="G23" s="10"/>
       <c r="H23" s="12"/>
       <c r="I23" s="5" t="s">
         <v>13</v>
@@ -1662,29 +1670,25 @@
       </c>
       <c r="M23" s="10"/>
       <c r="N23" s="12"/>
-      <c r="O23" s="22" t="s">
+      <c r="O23" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="P23" s="22"/>
-      <c r="Q23" s="10">
-        <v>1</v>
-      </c>
-      <c r="R23" s="25"/>
+      <c r="P23" s="32"/>
+      <c r="Q23" s="10"/>
+      <c r="R23" s="37"/>
       <c r="S23" s="12"/>
-      <c r="T23" s="22" t="s">
+      <c r="T23" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="U23" s="22"/>
+      <c r="U23" s="32"/>
       <c r="V23" s="10"/>
-      <c r="W23" s="25"/>
+      <c r="W23" s="37"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B24" s="18">
-        <v>1</v>
-      </c>
+      <c r="B24" s="10"/>
       <c r="F24" s="5" t="s">
         <v>14</v>
       </c>
@@ -1700,21 +1704,19 @@
       </c>
       <c r="M24" s="10"/>
       <c r="N24" s="12"/>
-      <c r="O24" s="22" t="s">
+      <c r="O24" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="P24" s="22"/>
-      <c r="Q24" s="10">
-        <v>4608</v>
-      </c>
-      <c r="R24" s="25"/>
+      <c r="P24" s="32"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="37"/>
       <c r="S24" s="12"/>
-      <c r="T24" s="22" t="s">
+      <c r="T24" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="U24" s="22"/>
+      <c r="U24" s="32"/>
       <c r="V24" s="10"/>
-      <c r="W24" s="25"/>
+      <c r="W24" s="37"/>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
@@ -1729,38 +1731,32 @@
       <c r="I25" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="J25" s="10">
-        <v>1</v>
-      </c>
+      <c r="J25" s="10"/>
       <c r="K25" s="12"/>
       <c r="L25" s="5" t="s">
         <v>15</v>
       </c>
       <c r="M25" s="10"/>
       <c r="N25" s="12"/>
-      <c r="O25" s="22" t="s">
+      <c r="O25" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="P25" s="22"/>
-      <c r="Q25" s="10">
-        <v>0</v>
-      </c>
-      <c r="R25" s="25"/>
+      <c r="P25" s="32"/>
+      <c r="Q25" s="10"/>
+      <c r="R25" s="37"/>
       <c r="S25" s="12"/>
-      <c r="T25" s="22" t="s">
+      <c r="T25" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="U25" s="22"/>
+      <c r="U25" s="32"/>
       <c r="V25" s="10"/>
-      <c r="W25" s="25"/>
+      <c r="W25" s="37"/>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="18">
-        <v>7</v>
-      </c>
+      <c r="B26" s="10"/>
       <c r="F26" s="5" t="s">
         <v>16</v>
       </c>
@@ -1776,21 +1772,19 @@
       </c>
       <c r="M26" s="10"/>
       <c r="N26" s="12"/>
-      <c r="O26" s="21" t="s">
+      <c r="O26" s="33" t="s">
         <v>47</v>
       </c>
-      <c r="P26" s="21"/>
-      <c r="Q26" s="10">
-        <v>0</v>
-      </c>
-      <c r="R26" s="25"/>
+      <c r="P26" s="33"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="37"/>
       <c r="S26" s="12"/>
-      <c r="T26" s="22" t="s">
+      <c r="T26" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="U26" s="22"/>
+      <c r="U26" s="32"/>
       <c r="V26" s="10"/>
-      <c r="W26" s="25"/>
+      <c r="W26" s="37"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
@@ -1805,40 +1799,32 @@
       <c r="I27" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="J27" s="10">
-        <v>7</v>
-      </c>
+      <c r="J27" s="10"/>
       <c r="K27" s="12"/>
       <c r="L27" s="5" t="s">
         <v>17</v>
       </c>
       <c r="M27" s="10"/>
       <c r="N27" s="12"/>
-      <c r="O27" s="21" t="s">
+      <c r="O27" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="P27" s="21"/>
-      <c r="Q27" s="10">
-        <v>94</v>
-      </c>
-      <c r="R27" s="25"/>
+      <c r="P27" s="33"/>
+      <c r="Q27" s="10"/>
+      <c r="R27" s="37"/>
       <c r="S27" s="12"/>
-      <c r="T27" s="22" t="s">
+      <c r="T27" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="U27" s="22"/>
-      <c r="V27" s="10">
-        <v>1836</v>
-      </c>
-      <c r="W27" s="25"/>
+      <c r="U27" s="32"/>
+      <c r="V27" s="10"/>
+      <c r="W27" s="37"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B28" s="18">
-        <v>5</v>
-      </c>
+      <c r="B28" s="10"/>
       <c r="F28" s="5" t="s">
         <v>52</v>
       </c>
@@ -1854,21 +1840,19 @@
       </c>
       <c r="M28" s="10"/>
       <c r="N28" s="12"/>
-      <c r="O28" s="21" t="s">
+      <c r="O28" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="P28" s="21"/>
-      <c r="Q28" s="10">
-        <v>289</v>
-      </c>
-      <c r="R28" s="25"/>
+      <c r="P28" s="33"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="37"/>
       <c r="S28" s="12"/>
-      <c r="T28" s="22" t="s">
+      <c r="T28" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="U28" s="22"/>
+      <c r="U28" s="32"/>
       <c r="V28" s="10"/>
-      <c r="W28" s="25"/>
+      <c r="W28" s="37"/>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
@@ -1878,9 +1862,7 @@
       <c r="F29" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G29" s="10">
-        <v>5</v>
-      </c>
+      <c r="G29" s="10"/>
       <c r="H29" s="12"/>
       <c r="I29" s="5" t="s">
         <v>47</v>
@@ -1892,27 +1874,23 @@
       </c>
       <c r="M29" s="10"/>
       <c r="N29" s="12"/>
-      <c r="O29" s="21" t="s">
+      <c r="O29" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="P29" s="21"/>
-      <c r="Q29" s="10">
-        <v>40046</v>
-      </c>
-      <c r="R29" s="25"/>
+      <c r="P29" s="33"/>
+      <c r="Q29" s="10"/>
+      <c r="R29" s="37"/>
       <c r="S29" s="12"/>
-      <c r="T29" s="17"/>
-      <c r="U29" s="17"/>
+      <c r="T29" s="16"/>
+      <c r="U29" s="16"/>
       <c r="V29" s="10"/>
-      <c r="W29" s="25"/>
+      <c r="W29" s="37"/>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="18">
-        <v>214</v>
-      </c>
+      <c r="B30" s="10"/>
       <c r="F30" s="5" t="s">
         <v>48</v>
       </c>
@@ -1928,19 +1906,17 @@
       </c>
       <c r="M30" s="10"/>
       <c r="N30" s="12"/>
-      <c r="O30" s="21" t="s">
+      <c r="O30" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="P30" s="21"/>
-      <c r="Q30" s="10">
-        <v>1</v>
-      </c>
-      <c r="R30" s="25"/>
+      <c r="P30" s="33"/>
+      <c r="Q30" s="10"/>
+      <c r="R30" s="37"/>
       <c r="S30" s="12"/>
-      <c r="T30" s="17"/>
-      <c r="U30" s="17"/>
+      <c r="T30" s="16"/>
+      <c r="U30" s="16"/>
       <c r="V30" s="10"/>
-      <c r="W30" s="25"/>
+      <c r="W30" s="37"/>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
@@ -1950,40 +1926,29 @@
       <c r="F31" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="G31" s="10">
-        <f>71</f>
-        <v>71</v>
-      </c>
+      <c r="G31" s="10"/>
       <c r="H31" s="12"/>
       <c r="I31" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="J31" s="10">
-        <f>72</f>
-        <v>72</v>
-      </c>
+      <c r="J31" s="10"/>
       <c r="K31" s="12"/>
       <c r="L31" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="M31" s="10">
-        <f>71</f>
-        <v>71</v>
-      </c>
+      <c r="M31" s="10"/>
       <c r="N31" s="12"/>
-      <c r="O31" s="21" t="s">
+      <c r="O31" s="33" t="s">
         <v>52</v>
       </c>
-      <c r="P31" s="21"/>
-      <c r="Q31" s="10">
-        <v>0</v>
-      </c>
-      <c r="R31" s="25"/>
+      <c r="P31" s="33"/>
+      <c r="Q31" s="10"/>
+      <c r="R31" s="37"/>
       <c r="S31" s="12"/>
-      <c r="T31" s="17"/>
-      <c r="U31" s="17"/>
+      <c r="T31" s="16"/>
+      <c r="U31" s="16"/>
       <c r="V31" s="10"/>
-      <c r="W31" s="25"/>
+      <c r="W31" s="37"/>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
@@ -2005,27 +1970,25 @@
       </c>
       <c r="M32" s="10"/>
       <c r="N32" s="12"/>
-      <c r="O32" s="21" t="s">
+      <c r="O32" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="10">
-        <v>733</v>
-      </c>
-      <c r="R32" s="25"/>
+      <c r="P32" s="33"/>
+      <c r="Q32" s="10"/>
+      <c r="R32" s="37"/>
       <c r="S32" s="12"/>
-      <c r="T32" s="22" t="s">
+      <c r="T32" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="U32" s="22"/>
+      <c r="U32" s="32"/>
       <c r="V32" s="10"/>
-      <c r="W32" s="25"/>
+      <c r="W32" s="37"/>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B33" s="16"/>
+      <c r="B33" s="10"/>
       <c r="F33" s="5" t="s">
         <v>53</v>
       </c>
@@ -2041,29 +2004,25 @@
       </c>
       <c r="M33" s="10"/>
       <c r="N33" s="12"/>
-      <c r="O33" s="21" t="s">
+      <c r="O33" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="P33" s="21"/>
-      <c r="Q33" s="10">
-        <v>2</v>
-      </c>
-      <c r="R33" s="25"/>
+      <c r="P33" s="33"/>
+      <c r="Q33" s="10"/>
+      <c r="R33" s="37"/>
       <c r="S33" s="12"/>
-      <c r="T33" s="22" t="s">
+      <c r="T33" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="U33" s="22"/>
+      <c r="U33" s="32"/>
       <c r="V33" s="10"/>
-      <c r="W33" s="25"/>
+      <c r="W33" s="37"/>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B34" s="20">
-        <v>1</v>
-      </c>
+      <c r="B34" s="10"/>
       <c r="F34" s="5" t="s">
         <v>19</v>
       </c>
@@ -2079,33 +2038,29 @@
       </c>
       <c r="M34" s="10"/>
       <c r="N34" s="12"/>
-      <c r="O34" s="21" t="s">
+      <c r="O34" s="33" t="s">
         <v>53</v>
       </c>
-      <c r="P34" s="21"/>
-      <c r="Q34" s="10">
-        <v>1</v>
-      </c>
-      <c r="R34" s="25"/>
+      <c r="P34" s="33"/>
+      <c r="Q34" s="10"/>
+      <c r="R34" s="37"/>
       <c r="S34" s="12"/>
-      <c r="T34" s="22" t="s">
+      <c r="T34" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="U34" s="22"/>
+      <c r="U34" s="32"/>
       <c r="V34" s="10"/>
-      <c r="W34" s="25"/>
+      <c r="W34" s="37"/>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B35" s="28"/>
+      <c r="B35" s="10"/>
       <c r="F35" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="G35" s="10">
-        <v>1</v>
-      </c>
+      <c r="G35" s="10"/>
       <c r="H35" s="12"/>
       <c r="I35" s="5" t="s">
         <v>49</v>
@@ -2117,29 +2072,25 @@
       </c>
       <c r="M35" s="10"/>
       <c r="N35" s="12"/>
-      <c r="O35" s="21" t="s">
+      <c r="O35" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="P35" s="21"/>
-      <c r="Q35" s="10">
-        <v>34</v>
-      </c>
-      <c r="R35" s="25"/>
+      <c r="P35" s="33"/>
+      <c r="Q35" s="10"/>
+      <c r="R35" s="37"/>
       <c r="S35" s="12"/>
-      <c r="T35" s="22" t="s">
+      <c r="T35" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="U35" s="22"/>
+      <c r="U35" s="32"/>
       <c r="V35" s="10"/>
-      <c r="W35" s="25"/>
+      <c r="W35" s="37"/>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B36" s="18">
-        <v>1</v>
-      </c>
+      <c r="B36" s="10"/>
       <c r="F36" s="5" t="s">
         <v>20</v>
       </c>
@@ -2155,21 +2106,19 @@
       </c>
       <c r="M36" s="10"/>
       <c r="N36" s="12"/>
-      <c r="O36" s="21" t="s">
+      <c r="O36" s="33" t="s">
         <v>49</v>
       </c>
-      <c r="P36" s="21"/>
-      <c r="Q36" s="10">
-        <v>10</v>
-      </c>
-      <c r="R36" s="25"/>
+      <c r="P36" s="33"/>
+      <c r="Q36" s="10"/>
+      <c r="R36" s="37"/>
       <c r="S36" s="12"/>
-      <c r="T36" s="22" t="s">
+      <c r="T36" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="U36" s="22"/>
+      <c r="U36" s="32"/>
       <c r="V36" s="10"/>
-      <c r="W36" s="25"/>
+      <c r="W36" s="37"/>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
@@ -2179,9 +2128,7 @@
       <c r="F37" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="G37" s="10">
-        <v>1</v>
-      </c>
+      <c r="G37" s="10"/>
       <c r="H37" s="12"/>
       <c r="I37" s="5" t="s">
         <v>21</v>
@@ -2193,19 +2140,17 @@
       </c>
       <c r="M37" s="10"/>
       <c r="N37" s="12"/>
-      <c r="O37" s="21" t="s">
+      <c r="O37" s="33" t="s">
         <v>59</v>
       </c>
-      <c r="P37" s="21"/>
-      <c r="Q37" s="10">
-        <v>1</v>
-      </c>
-      <c r="R37" s="25"/>
+      <c r="P37" s="33"/>
+      <c r="Q37" s="10"/>
+      <c r="R37" s="37"/>
       <c r="S37" s="12"/>
-      <c r="T37" s="19"/>
-      <c r="U37" s="19"/>
+      <c r="T37" s="17"/>
+      <c r="U37" s="17"/>
       <c r="V37" s="10"/>
-      <c r="W37" s="25"/>
+      <c r="W37" s="37"/>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
@@ -2227,27 +2172,23 @@
       </c>
       <c r="M38" s="10"/>
       <c r="N38" s="12"/>
-      <c r="O38" s="21" t="s">
+      <c r="O38" s="33" t="s">
         <v>60</v>
       </c>
-      <c r="P38" s="21"/>
-      <c r="Q38" s="10">
-        <v>2729</v>
-      </c>
-      <c r="R38" s="25"/>
+      <c r="P38" s="33"/>
+      <c r="Q38" s="10"/>
+      <c r="R38" s="37"/>
       <c r="S38" s="12"/>
-      <c r="T38" s="19"/>
-      <c r="U38" s="19"/>
+      <c r="T38" s="17"/>
+      <c r="U38" s="17"/>
       <c r="V38" s="10"/>
-      <c r="W38" s="25"/>
+      <c r="W38" s="37"/>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B39" s="18">
-        <v>17</v>
-      </c>
+      <c r="B39" s="10"/>
       <c r="F39" s="5" t="s">
         <v>23</v>
       </c>
@@ -2263,19 +2204,17 @@
       </c>
       <c r="M39" s="10"/>
       <c r="N39" s="12"/>
-      <c r="O39" s="21" t="s">
+      <c r="O39" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="P39" s="21"/>
-      <c r="Q39" s="10">
-        <v>34</v>
-      </c>
-      <c r="R39" s="25"/>
+      <c r="P39" s="33"/>
+      <c r="Q39" s="10"/>
+      <c r="R39" s="37"/>
       <c r="S39" s="12"/>
-      <c r="T39" s="19"/>
-      <c r="U39" s="19"/>
+      <c r="T39" s="17"/>
+      <c r="U39" s="17"/>
       <c r="V39" s="10"/>
-      <c r="W39" s="25"/>
+      <c r="W39" s="37"/>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
@@ -2290,30 +2229,24 @@
       <c r="I40" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="J40" s="10">
-        <v>8</v>
-      </c>
+      <c r="J40" s="10"/>
       <c r="K40" s="12"/>
       <c r="L40" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="M40" s="10">
-        <v>9</v>
-      </c>
+      <c r="M40" s="10"/>
       <c r="N40" s="12"/>
-      <c r="O40" s="21" t="s">
+      <c r="O40" s="33" t="s">
         <v>54</v>
       </c>
-      <c r="P40" s="21"/>
-      <c r="Q40" s="10">
-        <v>152</v>
-      </c>
-      <c r="R40" s="25"/>
+      <c r="P40" s="33"/>
+      <c r="Q40" s="10"/>
+      <c r="R40" s="37"/>
       <c r="S40" s="12"/>
-      <c r="T40" s="19"/>
-      <c r="U40" s="19"/>
+      <c r="T40" s="17"/>
+      <c r="U40" s="17"/>
       <c r="V40" s="10"/>
-      <c r="W40" s="25"/>
+      <c r="W40" s="37"/>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
@@ -2333,19 +2266,17 @@
       </c>
       <c r="M41" s="10"/>
       <c r="N41" s="12"/>
-      <c r="O41" s="21" t="s">
+      <c r="O41" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="P41" s="21"/>
-      <c r="Q41" s="10">
-        <v>10</v>
-      </c>
-      <c r="R41" s="25"/>
+      <c r="P41" s="33"/>
+      <c r="Q41" s="10"/>
+      <c r="R41" s="37"/>
       <c r="S41" s="12"/>
-      <c r="T41" s="19"/>
-      <c r="U41" s="19"/>
+      <c r="T41" s="17"/>
+      <c r="U41" s="17"/>
       <c r="V41" s="10"/>
-      <c r="W41" s="25"/>
+      <c r="W41" s="37"/>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
@@ -2363,23 +2294,19 @@
       </c>
       <c r="M42" s="10"/>
       <c r="N42" s="12"/>
-      <c r="O42" s="21" t="s">
+      <c r="O42" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="P42" s="21"/>
-      <c r="Q42" s="10">
-        <v>98</v>
-      </c>
-      <c r="R42" s="25"/>
+      <c r="P42" s="33"/>
+      <c r="Q42" s="10"/>
+      <c r="R42" s="37"/>
       <c r="S42" s="12"/>
-      <c r="T42" s="22" t="s">
+      <c r="T42" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="U42" s="22"/>
-      <c r="V42" s="10">
-        <v>216</v>
-      </c>
-      <c r="W42" s="25"/>
+      <c r="U42" s="32"/>
+      <c r="V42" s="10"/>
+      <c r="W42" s="37"/>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
@@ -2389,7 +2316,7 @@
       </c>
       <c r="G43" s="7">
         <f>SUM(G3:G42)</f>
-        <v>203</v>
+        <v>0</v>
       </c>
       <c r="H43" s="12"/>
       <c r="I43" s="6" t="s">
@@ -2397,7 +2324,7 @@
       </c>
       <c r="J43" s="7">
         <f>SUM(J3:J42)</f>
-        <v>192</v>
+        <v>0</v>
       </c>
       <c r="K43" s="12"/>
       <c r="L43" s="6" t="s">
@@ -2405,24 +2332,22 @@
       </c>
       <c r="M43" s="7">
         <f>SUM(M3:M42)</f>
-        <v>183</v>
+        <v>0</v>
       </c>
       <c r="N43" s="12"/>
-      <c r="O43" s="21" t="s">
+      <c r="O43" s="33" t="s">
         <v>55</v>
       </c>
-      <c r="P43" s="21"/>
-      <c r="Q43" s="10">
-        <v>35</v>
-      </c>
-      <c r="R43" s="25"/>
+      <c r="P43" s="33"/>
+      <c r="Q43" s="10"/>
+      <c r="R43" s="37"/>
       <c r="S43" s="12"/>
-      <c r="T43" s="22" t="s">
+      <c r="T43" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="U43" s="22"/>
+      <c r="U43" s="32"/>
       <c r="V43" s="10"/>
-      <c r="W43" s="25"/>
+      <c r="W43" s="37"/>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
@@ -2430,14 +2355,14 @@
       </c>
       <c r="B44" s="9">
         <f>SUM(B2:B43)</f>
-        <v>578</v>
+        <v>0</v>
       </c>
       <c r="F44" s="8" t="s">
         <v>27</v>
       </c>
       <c r="G44" s="9">
         <f>G43+J43+M43</f>
-        <v>578</v>
+        <v>0</v>
       </c>
       <c r="H44" s="12"/>
       <c r="I44" s="12"/>
@@ -2446,17 +2371,17 @@
       <c r="L44" s="12"/>
       <c r="M44" s="12"/>
       <c r="N44" s="12"/>
-      <c r="O44" s="22"/>
-      <c r="P44" s="22"/>
+      <c r="O44" s="32"/>
+      <c r="P44" s="32"/>
       <c r="Q44" s="10"/>
-      <c r="R44" s="25"/>
+      <c r="R44" s="37"/>
       <c r="S44" s="12"/>
-      <c r="T44" s="22" t="s">
+      <c r="T44" s="32" t="s">
         <v>22</v>
       </c>
-      <c r="U44" s="22"/>
+      <c r="U44" s="32"/>
       <c r="V44" s="10"/>
-      <c r="W44" s="25"/>
+      <c r="W44" s="37"/>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="8"/>
@@ -2470,50 +2395,120 @@
       <c r="L45" s="12"/>
       <c r="M45" s="12"/>
       <c r="N45" s="12"/>
-      <c r="O45" s="22"/>
-      <c r="P45" s="22"/>
+      <c r="O45" s="32"/>
+      <c r="P45" s="32"/>
       <c r="Q45" s="10"/>
-      <c r="R45" s="25"/>
+      <c r="R45" s="37"/>
       <c r="S45" s="12"/>
       <c r="T45" s="13"/>
       <c r="U45" s="13"/>
       <c r="V45" s="10"/>
-      <c r="W45" s="25"/>
+      <c r="W45" s="37"/>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O46" s="22"/>
-      <c r="P46" s="22"/>
+      <c r="O46" s="32"/>
+      <c r="P46" s="32"/>
       <c r="Q46" s="10"/>
-      <c r="R46" s="25"/>
-      <c r="T46" s="22" t="s">
+      <c r="R46" s="37"/>
+      <c r="T46" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="U46" s="22"/>
+      <c r="U46" s="32"/>
       <c r="V46" s="10"/>
-      <c r="W46" s="25"/>
+      <c r="W46" s="37"/>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O47" s="22"/>
-      <c r="P47" s="22"/>
+      <c r="O47" s="32"/>
+      <c r="P47" s="32"/>
       <c r="Q47" s="10"/>
-      <c r="R47" s="25"/>
-      <c r="T47" s="22" t="s">
+      <c r="R47" s="37"/>
+      <c r="T47" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="U47" s="22"/>
+      <c r="U47" s="32"/>
       <c r="V47" s="10"/>
-      <c r="W47" s="25"/>
+      <c r="W47" s="37"/>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="O48" s="23"/>
-      <c r="P48" s="23"/>
+      <c r="O48" s="38"/>
+      <c r="P48" s="38"/>
     </row>
     <row r="49" spans="15:16" x14ac:dyDescent="0.25">
-      <c r="O49" s="23"/>
-      <c r="P49" s="23"/>
+      <c r="O49" s="38"/>
+      <c r="P49" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="86">
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="O49:P49"/>
+    <mergeCell ref="O48:P48"/>
+    <mergeCell ref="O37:P37"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="O1:R1"/>
+    <mergeCell ref="R3:R47"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="O46:P46"/>
+    <mergeCell ref="O47:P47"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="O35:P35"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="O2:P2"/>
+    <mergeCell ref="O3:P3"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="T1:W1"/>
+    <mergeCell ref="T2:U2"/>
+    <mergeCell ref="T3:U3"/>
+    <mergeCell ref="W3:W47"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="T13:U13"/>
+    <mergeCell ref="T14:U14"/>
+    <mergeCell ref="T15:U15"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="T17:U17"/>
+    <mergeCell ref="T18:U18"/>
+    <mergeCell ref="T47:U47"/>
+    <mergeCell ref="T32:U32"/>
+    <mergeCell ref="T33:U33"/>
+    <mergeCell ref="T34:U34"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="T36:U36"/>
     <mergeCell ref="O7:P7"/>
     <mergeCell ref="T42:U42"/>
     <mergeCell ref="T43:U43"/>
@@ -2530,97 +2525,1759 @@
     <mergeCell ref="T22:U22"/>
     <mergeCell ref="T23:U23"/>
     <mergeCell ref="O27:P27"/>
-    <mergeCell ref="T47:U47"/>
-    <mergeCell ref="T32:U32"/>
-    <mergeCell ref="T33:U33"/>
-    <mergeCell ref="T34:U34"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="T36:U36"/>
-    <mergeCell ref="T1:W1"/>
-    <mergeCell ref="T2:U2"/>
-    <mergeCell ref="T3:U3"/>
-    <mergeCell ref="W3:W47"/>
-    <mergeCell ref="T4:U4"/>
-    <mergeCell ref="T5:U5"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="T9:U9"/>
-    <mergeCell ref="T11:U11"/>
-    <mergeCell ref="T13:U13"/>
-    <mergeCell ref="T14:U14"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="T16:U16"/>
-    <mergeCell ref="T17:U17"/>
-    <mergeCell ref="T18:U18"/>
-    <mergeCell ref="O2:P2"/>
-    <mergeCell ref="O3:P3"/>
-    <mergeCell ref="O4:P4"/>
-    <mergeCell ref="O5:P5"/>
-    <mergeCell ref="O6:P6"/>
-    <mergeCell ref="O25:P25"/>
-    <mergeCell ref="O26:P26"/>
-    <mergeCell ref="O21:P21"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="O12:P12"/>
-    <mergeCell ref="O1:R1"/>
-    <mergeCell ref="R3:R47"/>
-    <mergeCell ref="O43:P43"/>
-    <mergeCell ref="O44:P44"/>
-    <mergeCell ref="O46:P46"/>
-    <mergeCell ref="O47:P47"/>
-    <mergeCell ref="O28:P28"/>
-    <mergeCell ref="O32:P32"/>
-    <mergeCell ref="O33:P33"/>
-    <mergeCell ref="O34:P34"/>
-    <mergeCell ref="O35:P35"/>
-    <mergeCell ref="O36:P36"/>
-    <mergeCell ref="O22:P22"/>
-    <mergeCell ref="O23:P23"/>
-    <mergeCell ref="O24:P24"/>
-    <mergeCell ref="O29:P29"/>
-    <mergeCell ref="O30:P30"/>
-    <mergeCell ref="O31:P31"/>
-    <mergeCell ref="O45:P45"/>
-    <mergeCell ref="O49:P49"/>
-    <mergeCell ref="O48:P48"/>
-    <mergeCell ref="O37:P37"/>
-    <mergeCell ref="O38:P38"/>
-    <mergeCell ref="O39:P39"/>
-    <mergeCell ref="O40:P40"/>
-    <mergeCell ref="O41:P41"/>
-    <mergeCell ref="O42:P42"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.23622047244094491" right="0" top="0.35433070866141736" bottom="0.35433070866141736" header="0.31496062992125984" footer="0.31496062992125984"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="91" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:W48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <cols>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.42578125" customWidth="1"/>
+    <col min="5" max="5" width="9" customWidth="1"/>
+    <col min="6" max="6" width="9.140625" customWidth="1"/>
+    <col min="8" max="8" width="6.140625" customWidth="1"/>
+    <col min="11" max="11" width="5.28515625" customWidth="1"/>
+    <col min="18" max="18" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="6.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B1" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="42" t="s">
+        <v>56</v>
+      </c>
+      <c r="G1" s="42"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="42" t="s">
+        <v>57</v>
+      </c>
+      <c r="J1" s="42"/>
+      <c r="L1" s="42" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" s="42"/>
+      <c r="O1" s="44" t="s">
+        <v>62</v>
+      </c>
+      <c r="P1" s="44"/>
+      <c r="Q1" s="44"/>
+      <c r="R1" s="44"/>
+      <c r="T1" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+    </row>
+    <row r="2" spans="2:23" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="42"/>
+      <c r="J2" s="42"/>
+      <c r="L2" s="42"/>
+      <c r="M2" s="42"/>
+      <c r="O2" s="44"/>
+      <c r="P2" s="44"/>
+      <c r="Q2" s="44"/>
+      <c r="R2" s="44"/>
+      <c r="T2" s="42"/>
+      <c r="U2" s="42"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="42"/>
+    </row>
+    <row r="4" spans="2:23" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="45" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="39"/>
+      <c r="D4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="24"/>
+      <c r="F4" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="H4" s="26"/>
+      <c r="I4" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="J4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="K4" s="25"/>
+      <c r="L4" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="M4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="O4" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="R4" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="S4" s="25"/>
+      <c r="T4" s="43" t="s">
+        <v>0</v>
+      </c>
+      <c r="U4" s="43"/>
+      <c r="V4" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="W4" s="27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B5" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="18"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="19"/>
+      <c r="H5" s="25"/>
+      <c r="I5" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="J5" s="19"/>
+      <c r="K5" s="25"/>
+      <c r="L5" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="M5" s="19"/>
+      <c r="O5" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="P5" s="41"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="40">
+        <f>SUM(Q5:Q45)</f>
+        <v>0</v>
+      </c>
+      <c r="S5" s="25"/>
+      <c r="T5" s="41" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" s="41"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="40">
+        <f>SUM(V5:V45)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B6" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" s="19"/>
+      <c r="H6" s="25"/>
+      <c r="I6" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="J6" s="19"/>
+      <c r="K6" s="25"/>
+      <c r="L6" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="M6" s="19"/>
+      <c r="O6" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="P6" s="41"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="40"/>
+      <c r="S6" s="25"/>
+      <c r="T6" s="41" t="s">
+        <v>2</v>
+      </c>
+      <c r="U6" s="41"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="40"/>
+    </row>
+    <row r="7" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B7" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="18"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="25"/>
+      <c r="F7" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" s="19"/>
+      <c r="H7" s="25"/>
+      <c r="I7" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="J7" s="19"/>
+      <c r="K7" s="25"/>
+      <c r="L7" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="M7" s="19"/>
+      <c r="O7" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="P7" s="41"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="40"/>
+      <c r="S7" s="25"/>
+      <c r="T7" s="41" t="s">
+        <v>45</v>
+      </c>
+      <c r="U7" s="41"/>
+      <c r="V7" s="19"/>
+      <c r="W7" s="40"/>
+    </row>
+    <row r="8" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B8" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="G8" s="19"/>
+      <c r="H8" s="25"/>
+      <c r="I8" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="J8" s="19"/>
+      <c r="K8" s="25"/>
+      <c r="L8" s="18" t="s">
+        <v>3</v>
+      </c>
+      <c r="M8" s="19"/>
+      <c r="O8" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="P8" s="41"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="40"/>
+      <c r="S8" s="25"/>
+      <c r="T8" s="41" t="s">
+        <v>3</v>
+      </c>
+      <c r="U8" s="41"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="40"/>
+    </row>
+    <row r="9" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="25"/>
+      <c r="F9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="19"/>
+      <c r="H9" s="25"/>
+      <c r="I9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="M9" s="19"/>
+      <c r="O9" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="P9" s="41"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="40"/>
+      <c r="S9" s="25"/>
+      <c r="T9" s="41" t="s">
+        <v>50</v>
+      </c>
+      <c r="U9" s="41"/>
+      <c r="V9" s="19"/>
+      <c r="W9" s="40"/>
+    </row>
+    <row r="10" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="19"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="J10" s="19"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="18" t="s">
+        <v>44</v>
+      </c>
+      <c r="M10" s="19"/>
+      <c r="O10" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="P10" s="41"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="40"/>
+      <c r="S10" s="25"/>
+      <c r="T10" s="41" t="s">
+        <v>44</v>
+      </c>
+      <c r="U10" s="41"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="40"/>
+    </row>
+    <row r="11" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B11" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="25"/>
+      <c r="F11" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="19"/>
+      <c r="H11" s="25"/>
+      <c r="I11" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="18" t="s">
+        <v>33</v>
+      </c>
+      <c r="M11" s="19"/>
+      <c r="O11" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" s="41"/>
+      <c r="Q11" s="19"/>
+      <c r="R11" s="40"/>
+      <c r="S11" s="25"/>
+      <c r="T11" s="41" t="s">
+        <v>33</v>
+      </c>
+      <c r="U11" s="41"/>
+      <c r="V11" s="19"/>
+      <c r="W11" s="40"/>
+    </row>
+    <row r="12" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="25"/>
+      <c r="F12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="19"/>
+      <c r="H12" s="25"/>
+      <c r="I12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="J12" s="19"/>
+      <c r="K12" s="25"/>
+      <c r="L12" s="18" t="s">
+        <v>51</v>
+      </c>
+      <c r="M12" s="19"/>
+      <c r="O12" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="P12" s="41"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="40"/>
+      <c r="S12" s="25"/>
+      <c r="T12" s="41" t="s">
+        <v>51</v>
+      </c>
+      <c r="U12" s="41"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="40"/>
+    </row>
+    <row r="13" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B13" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+      <c r="E13" s="25"/>
+      <c r="F13" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="G13" s="19"/>
+      <c r="H13" s="25"/>
+      <c r="I13" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="J13" s="19"/>
+      <c r="K13" s="25"/>
+      <c r="L13" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="M13" s="19"/>
+      <c r="O13" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="P13" s="41"/>
+      <c r="Q13" s="19"/>
+      <c r="R13" s="40"/>
+      <c r="S13" s="25"/>
+      <c r="T13" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="U13" s="41"/>
+      <c r="V13" s="19"/>
+      <c r="W13" s="40"/>
+    </row>
+    <row r="14" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="19"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="J14" s="19"/>
+      <c r="K14" s="25"/>
+      <c r="L14" s="18" t="s">
+        <v>43</v>
+      </c>
+      <c r="M14" s="19"/>
+      <c r="O14" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="P14" s="41"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="40"/>
+      <c r="S14" s="25"/>
+      <c r="T14" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="U14" s="41"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="40"/>
+    </row>
+    <row r="15" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B15" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="19"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="J15" s="19"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="18" t="s">
+        <v>5</v>
+      </c>
+      <c r="M15" s="19"/>
+      <c r="O15" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="P15" s="41"/>
+      <c r="Q15" s="19"/>
+      <c r="R15" s="40"/>
+      <c r="S15" s="25"/>
+      <c r="T15" s="41" t="s">
+        <v>5</v>
+      </c>
+      <c r="U15" s="41"/>
+      <c r="V15" s="19"/>
+      <c r="W15" s="40"/>
+    </row>
+    <row r="16" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B16" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="19"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="G16" s="19"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="J16" s="19"/>
+      <c r="K16" s="25"/>
+      <c r="L16" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="M16" s="19"/>
+      <c r="O16" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="P16" s="41"/>
+      <c r="Q16" s="19"/>
+      <c r="R16" s="40"/>
+      <c r="S16" s="25"/>
+      <c r="T16" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="U16" s="41"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="40"/>
+    </row>
+    <row r="17" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" s="19"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="J17" s="19"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="M17" s="19"/>
+      <c r="O17" s="41" t="s">
+        <v>48</v>
+      </c>
+      <c r="P17" s="41"/>
+      <c r="Q17" s="19"/>
+      <c r="R17" s="40"/>
+      <c r="S17" s="25"/>
+      <c r="T17" s="41" t="s">
+        <v>48</v>
+      </c>
+      <c r="U17" s="41"/>
+      <c r="V17" s="19"/>
+      <c r="W17" s="40"/>
+    </row>
+    <row r="18" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" s="19"/>
+      <c r="H18" s="25"/>
+      <c r="I18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J18" s="19"/>
+      <c r="K18" s="25"/>
+      <c r="L18" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="M18" s="19"/>
+      <c r="O18" s="41" t="s">
+        <v>7</v>
+      </c>
+      <c r="P18" s="41"/>
+      <c r="Q18" s="19"/>
+      <c r="R18" s="40"/>
+      <c r="S18" s="25"/>
+      <c r="T18" s="41" t="s">
+        <v>7</v>
+      </c>
+      <c r="U18" s="41"/>
+      <c r="V18" s="19"/>
+      <c r="W18" s="40"/>
+    </row>
+    <row r="19" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" s="19"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" s="19"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="M19" s="19"/>
+      <c r="O19" s="41" t="s">
+        <v>8</v>
+      </c>
+      <c r="P19" s="41"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="40"/>
+      <c r="S19" s="25"/>
+      <c r="T19" s="41" t="s">
+        <v>8</v>
+      </c>
+      <c r="U19" s="41"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="40"/>
+    </row>
+    <row r="20" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B20" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="G20" s="19"/>
+      <c r="H20" s="25"/>
+      <c r="I20" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="J20" s="19"/>
+      <c r="K20" s="25"/>
+      <c r="L20" s="18" t="s">
+        <v>9</v>
+      </c>
+      <c r="M20" s="19"/>
+      <c r="O20" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="P20" s="41"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="40"/>
+      <c r="S20" s="25"/>
+      <c r="T20" s="41" t="s">
+        <v>9</v>
+      </c>
+      <c r="U20" s="41"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="40"/>
+    </row>
+    <row r="21" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="G21" s="19"/>
+      <c r="H21" s="25"/>
+      <c r="I21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="J21" s="19"/>
+      <c r="K21" s="25"/>
+      <c r="L21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M21" s="19"/>
+      <c r="O21" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="P21" s="41"/>
+      <c r="Q21" s="19"/>
+      <c r="R21" s="40"/>
+      <c r="S21" s="25"/>
+      <c r="T21" s="41" t="s">
+        <v>36</v>
+      </c>
+      <c r="U21" s="41"/>
+      <c r="V21" s="19"/>
+      <c r="W21" s="40"/>
+    </row>
+    <row r="22" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B22" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="C22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="19"/>
+      <c r="H22" s="25"/>
+      <c r="I22" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="J22" s="19"/>
+      <c r="K22" s="25"/>
+      <c r="L22" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="M22" s="19"/>
+      <c r="O22" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="P22" s="41"/>
+      <c r="Q22" s="19"/>
+      <c r="R22" s="40"/>
+      <c r="S22" s="25"/>
+      <c r="T22" s="41" t="s">
+        <v>10</v>
+      </c>
+      <c r="U22" s="41"/>
+      <c r="V22" s="19"/>
+      <c r="W22" s="40"/>
+    </row>
+    <row r="23" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B23" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="G23" s="19"/>
+      <c r="H23" s="25"/>
+      <c r="I23" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="J23" s="19"/>
+      <c r="K23" s="25"/>
+      <c r="L23" s="18" t="s">
+        <v>37</v>
+      </c>
+      <c r="M23" s="19"/>
+      <c r="O23" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="P23" s="41"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="40"/>
+      <c r="S23" s="25"/>
+      <c r="T23" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="U23" s="41"/>
+      <c r="V23" s="19"/>
+      <c r="W23" s="40"/>
+    </row>
+    <row r="24" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B24" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="25"/>
+      <c r="F24" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" s="19"/>
+      <c r="H24" s="25"/>
+      <c r="I24" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J24" s="19"/>
+      <c r="K24" s="25"/>
+      <c r="L24" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="M24" s="19"/>
+      <c r="O24" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="P24" s="41"/>
+      <c r="Q24" s="19"/>
+      <c r="R24" s="40"/>
+      <c r="S24" s="25"/>
+      <c r="T24" s="41" t="s">
+        <v>11</v>
+      </c>
+      <c r="U24" s="41"/>
+      <c r="V24" s="19"/>
+      <c r="W24" s="40"/>
+    </row>
+    <row r="25" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B25" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="25"/>
+      <c r="F25" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="G25" s="19"/>
+      <c r="H25" s="25"/>
+      <c r="I25" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="J25" s="19"/>
+      <c r="K25" s="25"/>
+      <c r="L25" s="18" t="s">
+        <v>38</v>
+      </c>
+      <c r="M25" s="19"/>
+      <c r="O25" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="P25" s="41"/>
+      <c r="Q25" s="19"/>
+      <c r="R25" s="40"/>
+      <c r="S25" s="25"/>
+      <c r="T25" s="41" t="s">
+        <v>38</v>
+      </c>
+      <c r="U25" s="41"/>
+      <c r="V25" s="19"/>
+      <c r="W25" s="40"/>
+    </row>
+    <row r="26" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B26" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="19"/>
+      <c r="E26" s="25"/>
+      <c r="F26" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="G26" s="19"/>
+      <c r="H26" s="25"/>
+      <c r="I26" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="J26" s="19"/>
+      <c r="K26" s="25"/>
+      <c r="L26" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="M26" s="19"/>
+      <c r="O26" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="P26" s="41"/>
+      <c r="Q26" s="19"/>
+      <c r="R26" s="40"/>
+      <c r="S26" s="25"/>
+      <c r="T26" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="U26" s="41"/>
+      <c r="V26" s="19"/>
+      <c r="W26" s="40"/>
+    </row>
+    <row r="27" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B27" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="18"/>
+      <c r="D27" s="19"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="19"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="J27" s="19"/>
+      <c r="K27" s="25"/>
+      <c r="L27" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="M27" s="19"/>
+      <c r="O27" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="P27" s="41"/>
+      <c r="Q27" s="19"/>
+      <c r="R27" s="40"/>
+      <c r="S27" s="25"/>
+      <c r="T27" s="41" t="s">
+        <v>13</v>
+      </c>
+      <c r="U27" s="41"/>
+      <c r="V27" s="19"/>
+      <c r="W27" s="40"/>
+    </row>
+    <row r="28" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B28" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="19"/>
+      <c r="E28" s="25"/>
+      <c r="F28" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="G28" s="19"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="J28" s="19"/>
+      <c r="K28" s="25"/>
+      <c r="L28" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="M28" s="19"/>
+      <c r="O28" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="P28" s="39"/>
+      <c r="Q28" s="19"/>
+      <c r="R28" s="40"/>
+      <c r="S28" s="25"/>
+      <c r="T28" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="U28" s="39"/>
+      <c r="V28" s="19"/>
+      <c r="W28" s="40"/>
+    </row>
+    <row r="29" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="18"/>
+      <c r="D29" s="19"/>
+      <c r="E29" s="25"/>
+      <c r="F29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" s="19"/>
+      <c r="H29" s="25"/>
+      <c r="I29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" s="19"/>
+      <c r="K29" s="25"/>
+      <c r="L29" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="M29" s="19"/>
+      <c r="O29" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="P29" s="39"/>
+      <c r="Q29" s="19"/>
+      <c r="R29" s="40"/>
+      <c r="S29" s="25"/>
+      <c r="T29" s="39" t="s">
+        <v>14</v>
+      </c>
+      <c r="U29" s="39"/>
+      <c r="V29" s="19"/>
+      <c r="W29" s="40"/>
+    </row>
+    <row r="30" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="18"/>
+      <c r="D30" s="19"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="G30" s="19"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="J30" s="19"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="M30" s="19"/>
+      <c r="O30" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="P30" s="39"/>
+      <c r="Q30" s="19"/>
+      <c r="R30" s="40"/>
+      <c r="S30" s="25"/>
+      <c r="T30" s="39" t="s">
+        <v>15</v>
+      </c>
+      <c r="U30" s="39"/>
+      <c r="V30" s="19"/>
+      <c r="W30" s="40"/>
+    </row>
+    <row r="31" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="18"/>
+      <c r="D31" s="19"/>
+      <c r="E31" s="25"/>
+      <c r="F31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="G31" s="19"/>
+      <c r="H31" s="25"/>
+      <c r="I31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="19"/>
+      <c r="K31" s="25"/>
+      <c r="L31" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="M31" s="19"/>
+      <c r="O31" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="P31" s="39"/>
+      <c r="Q31" s="19"/>
+      <c r="R31" s="40"/>
+      <c r="S31" s="25"/>
+      <c r="T31" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="U31" s="39"/>
+      <c r="V31" s="19"/>
+      <c r="W31" s="40"/>
+    </row>
+    <row r="32" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="25"/>
+      <c r="F32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="19"/>
+      <c r="H32" s="25"/>
+      <c r="I32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="J32" s="19"/>
+      <c r="K32" s="25"/>
+      <c r="L32" s="18" t="s">
+        <v>17</v>
+      </c>
+      <c r="M32" s="19"/>
+      <c r="O32" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="P32" s="39"/>
+      <c r="Q32" s="19"/>
+      <c r="R32" s="40"/>
+      <c r="S32" s="25"/>
+      <c r="T32" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="U32" s="39"/>
+      <c r="V32" s="19"/>
+      <c r="W32" s="40"/>
+    </row>
+    <row r="33" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B33" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C33" s="18"/>
+      <c r="D33" s="19"/>
+      <c r="E33" s="25"/>
+      <c r="F33" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G33" s="19"/>
+      <c r="H33" s="25"/>
+      <c r="I33" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="J33" s="19"/>
+      <c r="K33" s="25"/>
+      <c r="L33" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="M33" s="19"/>
+      <c r="O33" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="P33" s="39"/>
+      <c r="Q33" s="19"/>
+      <c r="R33" s="40"/>
+      <c r="S33" s="25"/>
+      <c r="T33" s="39" t="s">
+        <v>52</v>
+      </c>
+      <c r="U33" s="39"/>
+      <c r="V33" s="19"/>
+      <c r="W33" s="40"/>
+    </row>
+    <row r="34" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B34" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="18"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="G34" s="19"/>
+      <c r="H34" s="25"/>
+      <c r="I34" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="J34" s="19"/>
+      <c r="K34" s="25"/>
+      <c r="L34" s="18" t="s">
+        <v>18</v>
+      </c>
+      <c r="M34" s="19"/>
+      <c r="O34" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="P34" s="39"/>
+      <c r="Q34" s="31"/>
+      <c r="R34" s="40"/>
+      <c r="S34" s="25"/>
+      <c r="T34" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="U34" s="39"/>
+      <c r="V34" s="19"/>
+      <c r="W34" s="40"/>
+    </row>
+    <row r="35" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B35" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C35" s="18"/>
+      <c r="D35" s="19"/>
+      <c r="E35" s="25"/>
+      <c r="F35" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="G35" s="19"/>
+      <c r="H35" s="25"/>
+      <c r="I35" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="J35" s="19"/>
+      <c r="K35" s="25"/>
+      <c r="L35" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="M35" s="19"/>
+      <c r="O35" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="P35" s="39"/>
+      <c r="Q35" s="19"/>
+      <c r="R35" s="40"/>
+      <c r="S35" s="25"/>
+      <c r="T35" s="39" t="s">
+        <v>46</v>
+      </c>
+      <c r="U35" s="39"/>
+      <c r="V35" s="19"/>
+      <c r="W35" s="40"/>
+    </row>
+    <row r="36" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B36" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="C36" s="18"/>
+      <c r="D36" s="19"/>
+      <c r="E36" s="25"/>
+      <c r="F36" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G36" s="19"/>
+      <c r="H36" s="25"/>
+      <c r="I36" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="J36" s="19"/>
+      <c r="K36" s="25"/>
+      <c r="L36" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="M36" s="19"/>
+      <c r="O36" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="P36" s="39"/>
+      <c r="Q36" s="19"/>
+      <c r="R36" s="40"/>
+      <c r="S36" s="25"/>
+      <c r="T36" s="39" t="s">
+        <v>53</v>
+      </c>
+      <c r="U36" s="39"/>
+      <c r="V36" s="19"/>
+      <c r="W36" s="40"/>
+    </row>
+    <row r="37" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B37" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="C37" s="18"/>
+      <c r="D37" s="19"/>
+      <c r="E37" s="25"/>
+      <c r="F37" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="G37" s="19"/>
+      <c r="H37" s="25"/>
+      <c r="I37" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="J37" s="19"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="M37" s="19"/>
+      <c r="O37" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="P37" s="39"/>
+      <c r="Q37" s="19"/>
+      <c r="R37" s="40"/>
+      <c r="S37" s="25"/>
+      <c r="T37" s="39" t="s">
+        <v>19</v>
+      </c>
+      <c r="U37" s="39"/>
+      <c r="V37" s="19"/>
+      <c r="W37" s="40"/>
+    </row>
+    <row r="38" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B38" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="25"/>
+      <c r="F38" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="G38" s="19"/>
+      <c r="H38" s="25"/>
+      <c r="I38" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="J38" s="19"/>
+      <c r="K38" s="25"/>
+      <c r="L38" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="M38" s="19"/>
+      <c r="O38" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="P38" s="39"/>
+      <c r="Q38" s="19"/>
+      <c r="R38" s="40"/>
+      <c r="S38" s="25"/>
+      <c r="T38" s="39" t="s">
+        <v>49</v>
+      </c>
+      <c r="U38" s="39"/>
+      <c r="V38" s="19"/>
+      <c r="W38" s="40"/>
+    </row>
+    <row r="39" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B39" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" s="18"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="G39" s="19"/>
+      <c r="H39" s="25"/>
+      <c r="I39" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="J39" s="19"/>
+      <c r="K39" s="25"/>
+      <c r="L39" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="M39" s="19"/>
+      <c r="O39" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="P39" s="39"/>
+      <c r="Q39" s="19"/>
+      <c r="R39" s="40"/>
+      <c r="S39" s="25"/>
+      <c r="T39" s="39" t="s">
+        <v>59</v>
+      </c>
+      <c r="U39" s="39"/>
+      <c r="V39" s="19"/>
+      <c r="W39" s="40"/>
+    </row>
+    <row r="40" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" s="18"/>
+      <c r="D40" s="19"/>
+      <c r="E40" s="25"/>
+      <c r="F40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="G40" s="19"/>
+      <c r="H40" s="25"/>
+      <c r="I40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="J40" s="19"/>
+      <c r="K40" s="25"/>
+      <c r="L40" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="M40" s="19"/>
+      <c r="O40" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="P40" s="39"/>
+      <c r="Q40" s="19"/>
+      <c r="R40" s="40"/>
+      <c r="S40" s="25"/>
+      <c r="T40" s="39" t="s">
+        <v>60</v>
+      </c>
+      <c r="U40" s="39"/>
+      <c r="V40" s="19"/>
+      <c r="W40" s="40"/>
+    </row>
+    <row r="41" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B41" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="18"/>
+      <c r="D41" s="19"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="19"/>
+      <c r="H41" s="25"/>
+      <c r="I41" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="J41" s="19"/>
+      <c r="K41" s="25"/>
+      <c r="L41" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="M41" s="19"/>
+      <c r="O41" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="P41" s="39"/>
+      <c r="Q41" s="19"/>
+      <c r="R41" s="40"/>
+      <c r="S41" s="25"/>
+      <c r="T41" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="U41" s="39"/>
+      <c r="V41" s="19"/>
+      <c r="W41" s="40"/>
+    </row>
+    <row r="42" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B42" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C42" s="18"/>
+      <c r="D42" s="19"/>
+      <c r="E42" s="25"/>
+      <c r="F42" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="G42" s="19"/>
+      <c r="H42" s="25"/>
+      <c r="I42" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="J42" s="19"/>
+      <c r="K42" s="25"/>
+      <c r="L42" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="M42" s="19"/>
+      <c r="O42" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="P42" s="39"/>
+      <c r="Q42" s="19"/>
+      <c r="R42" s="40"/>
+      <c r="S42" s="25"/>
+      <c r="T42" s="39" t="s">
+        <v>54</v>
+      </c>
+      <c r="U42" s="39"/>
+      <c r="V42" s="19"/>
+      <c r="W42" s="40"/>
+    </row>
+    <row r="43" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="C43" s="18"/>
+      <c r="D43" s="19"/>
+      <c r="E43" s="25"/>
+      <c r="F43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G43" s="19"/>
+      <c r="H43" s="25"/>
+      <c r="I43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="J43" s="19"/>
+      <c r="K43" s="25"/>
+      <c r="L43" s="18" t="s">
+        <v>23</v>
+      </c>
+      <c r="M43" s="19"/>
+      <c r="O43" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="P43" s="39"/>
+      <c r="Q43" s="19"/>
+      <c r="R43" s="40"/>
+      <c r="S43" s="25"/>
+      <c r="T43" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="U43" s="39"/>
+      <c r="V43" s="19"/>
+      <c r="W43" s="40"/>
+    </row>
+    <row r="44" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B44" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C44" s="18"/>
+      <c r="D44" s="19"/>
+      <c r="E44" s="25"/>
+      <c r="F44" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="G44" s="19"/>
+      <c r="H44" s="25"/>
+      <c r="I44" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="J44" s="19"/>
+      <c r="K44" s="25"/>
+      <c r="L44" s="18" t="s">
+        <v>24</v>
+      </c>
+      <c r="M44" s="19"/>
+      <c r="O44" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="P44" s="39"/>
+      <c r="Q44" s="19"/>
+      <c r="R44" s="40"/>
+      <c r="S44" s="25"/>
+      <c r="T44" s="39" t="s">
+        <v>24</v>
+      </c>
+      <c r="U44" s="39"/>
+      <c r="V44" s="19"/>
+      <c r="W44" s="40"/>
+    </row>
+    <row r="45" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B45" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="C45" s="18"/>
+      <c r="D45" s="19"/>
+      <c r="E45" s="25"/>
+      <c r="F45" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="G45" s="19"/>
+      <c r="H45" s="25"/>
+      <c r="I45" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="J45" s="19"/>
+      <c r="K45" s="25"/>
+      <c r="L45" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="M45" s="19"/>
+      <c r="O45" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="P45" s="39"/>
+      <c r="Q45" s="19"/>
+      <c r="R45" s="40"/>
+      <c r="S45" s="25"/>
+      <c r="T45" s="39" t="s">
+        <v>55</v>
+      </c>
+      <c r="U45" s="39"/>
+      <c r="V45" s="19"/>
+      <c r="W45" s="40"/>
+    </row>
+    <row r="46" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B46" s="18"/>
+      <c r="C46" s="18"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="25"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="19"/>
+      <c r="H46" s="25"/>
+      <c r="I46" s="18"/>
+      <c r="J46" s="19"/>
+      <c r="K46" s="25"/>
+      <c r="L46" s="18"/>
+      <c r="M46" s="19"/>
+      <c r="O46" s="18"/>
+      <c r="P46" s="18"/>
+      <c r="Q46" s="19"/>
+      <c r="R46" s="40"/>
+      <c r="S46" s="25"/>
+      <c r="T46" s="18"/>
+      <c r="U46" s="18"/>
+      <c r="V46" s="19"/>
+      <c r="W46" s="40"/>
+    </row>
+    <row r="47" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B47" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C47" s="29">
+        <v>0</v>
+      </c>
+      <c r="D47" s="19"/>
+      <c r="E47" s="25"/>
+      <c r="F47" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="G47" s="30">
+        <f>SUM(G5:G45)</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="25"/>
+      <c r="I47" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="J47" s="30">
+        <f>SUM(J5:J45)</f>
+        <v>0</v>
+      </c>
+      <c r="K47" s="25"/>
+      <c r="L47" s="28" t="s">
+        <v>26</v>
+      </c>
+      <c r="M47" s="30">
+        <f>SUM(M5:M45)</f>
+        <v>0</v>
+      </c>
+      <c r="O47" s="18"/>
+      <c r="P47" s="18"/>
+      <c r="Q47" s="19"/>
+      <c r="R47" s="40"/>
+      <c r="S47" s="25"/>
+      <c r="T47" s="18"/>
+      <c r="U47" s="18"/>
+      <c r="V47" s="19"/>
+      <c r="W47" s="40"/>
+    </row>
+    <row r="48" spans="2:23" x14ac:dyDescent="0.25">
+      <c r="B48" s="18"/>
+      <c r="C48" s="18"/>
+      <c r="D48" s="19"/>
+      <c r="E48" s="25"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="19"/>
+      <c r="H48" s="25"/>
+      <c r="I48" s="18"/>
+      <c r="J48" s="19"/>
+      <c r="K48" s="25"/>
+      <c r="L48" s="18"/>
+      <c r="M48" s="19"/>
+      <c r="O48" s="18"/>
+      <c r="P48" s="18"/>
+      <c r="Q48" s="19"/>
+      <c r="R48" s="40"/>
+      <c r="S48" s="25"/>
+      <c r="T48" s="18"/>
+      <c r="U48" s="18"/>
+      <c r="V48" s="19"/>
+      <c r="W48" s="40"/>
+    </row>
+  </sheetData>
+  <mergeCells count="93">
+    <mergeCell ref="B1:D2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="F1:G2"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="I1:J2"/>
+    <mergeCell ref="L1:M2"/>
+    <mergeCell ref="O1:R2"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="O6:P6"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="O22:P22"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O37:P37"/>
+    <mergeCell ref="O38:P38"/>
+    <mergeCell ref="O39:P39"/>
+    <mergeCell ref="O40:P40"/>
+    <mergeCell ref="O29:P29"/>
+    <mergeCell ref="O30:P30"/>
+    <mergeCell ref="O31:P31"/>
+    <mergeCell ref="O32:P32"/>
+    <mergeCell ref="O33:P33"/>
+    <mergeCell ref="O34:P34"/>
+    <mergeCell ref="T1:W2"/>
+    <mergeCell ref="T4:U4"/>
+    <mergeCell ref="T5:U5"/>
+    <mergeCell ref="O35:P35"/>
+    <mergeCell ref="O36:P36"/>
+    <mergeCell ref="O23:P23"/>
+    <mergeCell ref="O24:P24"/>
+    <mergeCell ref="O25:P25"/>
+    <mergeCell ref="O26:P26"/>
+    <mergeCell ref="O27:P27"/>
+    <mergeCell ref="O28:P28"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="O21:P21"/>
+    <mergeCell ref="O41:P41"/>
+    <mergeCell ref="O42:P42"/>
+    <mergeCell ref="O43:P43"/>
+    <mergeCell ref="O44:P44"/>
+    <mergeCell ref="O45:P45"/>
+    <mergeCell ref="T14:U14"/>
+    <mergeCell ref="T15:U15"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="T17:U17"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="T9:U9"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="W5:W48"/>
+    <mergeCell ref="T36:U36"/>
+    <mergeCell ref="T37:U37"/>
+    <mergeCell ref="T38:U38"/>
+    <mergeCell ref="T39:U39"/>
+    <mergeCell ref="T40:U40"/>
+    <mergeCell ref="T41:U41"/>
+    <mergeCell ref="T30:U30"/>
+    <mergeCell ref="T31:U31"/>
+    <mergeCell ref="T32:U32"/>
+    <mergeCell ref="T33:U33"/>
+    <mergeCell ref="T34:U34"/>
+    <mergeCell ref="T35:U35"/>
+    <mergeCell ref="T24:U24"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="T26:U26"/>
+    <mergeCell ref="T42:U42"/>
+    <mergeCell ref="T43:U43"/>
+    <mergeCell ref="T44:U44"/>
+    <mergeCell ref="T45:U45"/>
+    <mergeCell ref="R5:R48"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="T28:U28"/>
+    <mergeCell ref="T29:U29"/>
+    <mergeCell ref="T18:U18"/>
+    <mergeCell ref="T19:U19"/>
+    <mergeCell ref="T20:U20"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="T22:U22"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="T12:U12"/>
+    <mergeCell ref="T13:U13"/>
+  </mergeCells>
+  <pageMargins left="0.15748031496062992" right="0.15748031496062992" top="0.15748031496062992" bottom="0.15748031496062992" header="0.31496062992125984" footer="0.31496062992125984"/>
+  <pageSetup paperSize="9" scale="70" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>